<commit_message>
Add chest valve and door
</commit_message>
<xml_diff>
--- a/Docs/TechDoc.xlsx
+++ b/Docs/TechDoc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UnityProject\Test_Ivanov_SnapJoy\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92DDFD9F-E216-4E2A-B551-DAAE4372605B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A5BE9A-924F-46CA-9C85-38C166C25EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="34560" windowHeight="19140" xr2:uid="{27FC311B-5DC4-4BD0-B18D-2A9521915081}"/>
+    <workbookView xWindow="2184" yWindow="3732" windowWidth="34560" windowHeight="19140" xr2:uid="{27FC311B-5DC4-4BD0-B18D-2A9521915081}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Создать контроллер игрока</t>
   </si>
@@ -36,10 +36,43 @@
     <t>Создать ситему взаимодействия с Interacltable Обьектом</t>
   </si>
   <si>
-    <t>у нас сейчас разграничены press И Hold</t>
-  </si>
-  <si>
     <t>Доп взаимодейстиивие взлом. Пусть у нас будет шифр указаный азбукой морзе который надо набить</t>
+  </si>
+  <si>
+    <t>для предмета это будет открыватель дверей. Он посылает код системе (есть в записке азбукой)</t>
+  </si>
+  <si>
+    <t>подобор предмета</t>
+  </si>
+  <si>
+    <t>расмотр предмета</t>
+  </si>
+  <si>
+    <t>книжка</t>
+  </si>
+  <si>
+    <t>сундук</t>
+  </si>
+  <si>
+    <t>набивание кода</t>
+  </si>
+  <si>
+    <t>предмет рушащий стену или толкающий НПС</t>
+  </si>
+  <si>
+    <t>вентиль</t>
+  </si>
+  <si>
+    <t>начало диалога с НПС</t>
+  </si>
+  <si>
+    <t>диалоги с НПС</t>
+  </si>
+  <si>
+    <t>НПС + квестовая лингия</t>
+  </si>
+  <si>
+    <t>ращложить по папкам + readme</t>
   </si>
 </sst>
 </file>
@@ -56,12 +89,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -76,8 +115,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -392,47 +433,138 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10C52446-75A4-42D3-9D37-18E78F600A99}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1">
+      <c r="B1" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="2">
+        <v>7</v>
+      </c>
+    </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>3</v>
+      <c r="A14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B10">
+    <sortCondition ref="B10"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>